<commit_message>
Plano de conexao: incorpora calendario de redes sociais da Gabriela (17 frentes, 11 marcos)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/plano-conexao-diretoria-2026-10-16.xlsx
+++ b/docs/nekt/plano-conexao-diretoria-2026-10-16.xlsx
@@ -529,14 +529,14 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Frentes: 15 frentes com prioridade, complexidade, dependências, responsável, prazo, frequência e créditos.</t>
+          <t>Frentes: 17 frentes com prioridade, complexidade, dependências, responsável, prazo, frequência e créditos.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Marcos: 9 marcos verificáveis e a cobertura esperada.</t>
+          <t>Marcos: 11 marcos verificáveis e a cobertura esperada.</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Decisão 23/10; fechamento 02/11</t>
+          <t>Instagram: conexão 20/10 (calendário da Gabriela); lista de contas e agenda 23/10; fechamento 02/11</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1503,50 +1503,164 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>TikTok orgânico (conector tiktok: perfil e vídeos; difere do TikTok Ads da F09)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>a definir (fora das 209)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Contas e acessos do TikTok orgânico por cliente; nome de camada confirmado (R-001); Trusted nova a criar</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Gabriela Bezerra + Jussara</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Conexão 21/10 a 23/10 (calendário da Gabriela)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>+4,35 por fonte (nº de fontes a definir)</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Fonte com 1ª execução agendada e linhas na tabela (27/10 se semanal na terça)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>F16</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Google Meu Negócio (conector google-my-business; sem fonte hoje)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>a definir (fora das 209)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Levantamento de contas e proprietários dos perfis; convites e permissões dos donos; Trusted nova a criar</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Gabriela Bezerra + Jussara</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Levantamento 26/10; conexão até 29/10; buffer 30/10</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>+4,35 por fonte (nº de fontes a definir)</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Fontes com 1ª execução agendada e linhas na tabela (03/11 se semanal na terça)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>Fechamento: relatório final de cobertura</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>209 contas</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>209 contas + frentes novas</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>F01 a F13</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>F01 a F16</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Jussara</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>04/11</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Cobertura recalculada com a mesma metodologia e entregue</t>
         </is>
@@ -1563,7 +1677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1651,7 +1765,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Passada de Meta e Google; nenhuma fonte desativada</t>
+          <t>Passada de Meta e Google; nenhuma fonte desativada. Gabriela finaliza a conexão do Instagram (calendário dela)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -1661,12 +1775,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>list_pipeline_runs: zero fonte desativada pela regra das 3 falhas; as 7 de 403 falham de novo (esperado)</t>
+          <t>list_pipeline_runs: zero fonte desativada pela regra das 3 falhas; as 7 de 403 falham de novo (esperado); fontes de Instagram com agenda definida</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Jussara</t>
+          <t>Jussara; Gabriela Bezerra</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1797,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Pedidos enviados e IDs Google levantados</t>
+          <t>Pedidos enviados e IDs Google levantados; início do TikTok orgânico</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1698,7 +1812,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Jussara; João Araújo</t>
+          <t>Jussara; João Araújo; Gabriela Bezerra</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1861,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Prazo duro do Google; decisões da Diretoria; lista de Instagram e Páginas</t>
+          <t>Prazo duro do Google; decisões da Diretoria; lista de Instagram e Páginas; TikTok orgânico validado (calendário da Gabriela)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1757,7 +1871,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Decisões registradas; lista de contas exigidas definida</t>
+          <t>Decisões registradas; lista de contas exigidas definida; conta TikTok orgânica integrada</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1779,7 +1893,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1ª execução agendada das 28 fontes publicadas; 8 contas Meta sem erro</t>
+          <t>1ª execução agendada das 28 fontes publicadas e do Instagram; 8 contas Meta sem erro</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1838,27 +1952,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>03/11 (terça)</t>
+          <t>29/10</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Contas novas na Trusted; TikTok e LinkedIn com 1ª execução; Instagram e Páginas fechados (02/11)</t>
+          <t>Google Meu Negócio finalizado e validado (calendário da Gabriela)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>até 209</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>LIMIT 0 na união; contas novas conferidas contra a plataforma (≤ 1%)</t>
+          <t>Permissões e integração das contas conferidas; fonte publicada</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Jussara; Gabriela Bezerra</t>
+          <t>Gabriela Bezerra</t>
         </is>
       </c>
     </row>
@@ -1870,25 +1984,89 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>30/10</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Buffer de redes sociais: ajustes finais de Instagram, TikTok e Google Meu Negócio; IDs de TikTok Ads e LinkedIn</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Pendências residuais registradas; status final das integrações consolidado</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Gabriela Bezerra; João Araújo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>03/11 (terça)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Contas novas na Trusted; TikTok Ads e LinkedIn com 1ª execução; Google Meu Negócio com 1ª execução; Instagram e Páginas fechados (02/11)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>até 209</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>LIMIT 0 na união; contas novas conferidas contra a plataforma (≤ 1%)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Jussara; Gabriela Bezerra</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>04/11</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Relatório final de cobertura e indicadores</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>209 de 209 (100%) se tudo for entregue; piso 204 (97,6%) se CDL e 3 contas Google de ID pendente ficarem de fora</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Mesma metodologia da linha de base</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Jussara</t>
         </is>
@@ -1905,7 +2083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2080,7 +2258,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>TikTok e LinkedIn</t>
+          <t>TikTok Ads e LinkedIn</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2107,100 +2285,111 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Instagram e Páginas (26 fontes)</t>
+          <t>TikTok orgânico e Google Meu Negócio</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Manuais</t>
+          <t>Sem fonte (conectores tiktok e google-my-business existem)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Semanal (diário custa +761)</t>
+          <t>Semanal</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>+118</t>
+          <t>+4,35 por fonte; nº de fontes a definir</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Extração mínima hoje: 0 a 9 posts por conta; lista de contas exigidas não existe</t>
+          <t>Fora das 209 contas aplicáveis; créditos acima dos +287 do plano</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Instagram e Páginas (26 fontes)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Manuais</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Semanal (diário custa +761)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>+118</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Extração mínima hoje: 0 a 9 posts por conta; lista de contas exigidas não existe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>GitHub, Z-API, Semrush, RH</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>GitHub semanal; Z-API diária; os demais sem fonte funcional</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Semanal</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>+13</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Só entram quando a fonte entregar dado</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Cenário</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Créditos por mês</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>% de 9.000</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Sem manuais, regra "todas"</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>7888</v>
-      </c>
-      <c r="C12" s="8">
-        <f>B12/9000</f>
-        <v/>
-      </c>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>300 manuais por mês, regra "todas"</t>
+          <t>Sem manuais, regra "todas"</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>8188</v>
+        <v>7888</v>
       </c>
       <c r="C13" s="8">
         <f>B13/9000</f>
@@ -2212,11 +2401,11 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Ritmo de outubro (≈ 1.200 manuais), regra "todas"</t>
+          <t>300 manuais por mês, regra "todas"</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>9088</v>
+        <v>8188</v>
       </c>
       <c r="C14" s="8">
         <f>B14/9000</f>
@@ -2228,11 +2417,11 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>300 manuais, regra "qualquer"</t>
+          <t>Ritmo de outubro (≈ 1.200 manuais), regra "todas"</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>8732</v>
+        <v>9088</v>
       </c>
       <c r="C15" s="8">
         <f>B15/9000</f>
@@ -2244,11 +2433,11 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Ritmo de outubro, regra "qualquer"</t>
+          <t>300 manuais, regra "qualquer"</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>9632</v>
+        <v>8732</v>
       </c>
       <c r="C16" s="8">
         <f>B16/9000</f>
@@ -2260,11 +2449,11 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Sem manuais, notebook do iClips em 8h (derivado: 7.888 − 1.650)</t>
+          <t>Ritmo de outubro, regra "qualquer"</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>6238</v>
+        <v>9632</v>
       </c>
       <c r="C17" s="8">
         <f>B17/9000</f>
@@ -2273,8 +2462,24 @@
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Sem manuais, notebook do iClips em 8h (derivado: 7.888 − 1.650)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>6238</v>
+      </c>
+      <c r="C18" s="8">
+        <f>B18/9000</f>
+        <v/>
+      </c>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Regra do crédito: 1 por execução bem-sucedida de fonte, consulta, notebook, histórico ou destino; falha e carga inicial de fonte não são cobradas. O consumo real não é legível pelo token (nekt_runs inacessível): conferir em Billing.</t>
         </is>

</xml_diff>